<commit_message>
feat: add optional view counts and field-level validation
</commit_message>
<xml_diff>
--- a/docs/数据库表结构.xlsx
+++ b/docs/数据库表结构.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="Rad431ca53a194ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="Re73aa3a8a85546c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="R12a560fadd504993"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="R4548d21c509940bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="Rfdfd868e68164c08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R1d11919ec92d44db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="R465926a4ea79427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="R40af13e9baa84f1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R04ff76e7f99a44f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="Rf32115cae53c40e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="Rce6898a1382b419e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="R48914bcd511f4443"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R8f708452330543ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="R2a743f640371496c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设计规则" sheetId="1" r:id="Rd40198d6f67f44f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="表清单" sheetId="2" r:id="R0239707e36184be2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user" sheetId="3" r:id="R2426dc62deb748b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role" sheetId="4" r:id="Rf4b784e5da244ec2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_role" sheetId="5" r:id="R237e65893a06434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_menu" sheetId="6" r:id="R56b778ce8e1f4972"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_role_menu" sheetId="7" r:id="R38dbdf9f249c4ed9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_work_order" sheetId="8" r:id="Rdcad48a3d8e94dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive_type" sheetId="9" r:id="R5a2e20d2154a47c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_archive" sheetId="10" r:id="R43b3fbbea4404882"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_op_log" sheetId="11" r:id="R24a613988c8b4a84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_access_log" sheetId="12" r:id="Rd03b6ad23d484af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_user_preference" sheetId="13" r:id="R63f0a904052e4e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pms_message" sheetId="14" r:id="Ra6082f9ea4f84b70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -645,9 +645,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">新员工账号权限开通</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">工单问题描述。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">处置结果</x:t>
@@ -2444,7 +2441,7 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>258</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -2520,13 +2517,13 @@
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A4" s="7" t="s">
-        <x:v>259</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="B4" s="7" t="s">
         <x:v>142</x:v>
       </x:c>
       <x:c r="C4" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D4" s="7" t="s">
         <x:v>90</x:v>
@@ -2540,21 +2537,21 @@
       </x:c>
       <x:c r="H4" s="7"/>
       <x:c r="I4" s="8" t="s">
+        <x:v>259</x:v>
+      </x:c>
+      <x:c r="J4" s="7" t="s">
         <x:v>260</x:v>
-      </x:c>
-      <x:c r="J4" s="7" t="s">
-        <x:v>261</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A5" s="7" t="s">
-        <x:v>262</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="B5" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D5" s="7" t="s">
         <x:v>90</x:v>
@@ -2564,18 +2561,18 @@
       <x:c r="G5" s="7"/>
       <x:c r="H5" s="7"/>
       <x:c r="I5" s="8" t="s">
+        <x:v>262</x:v>
+      </x:c>
+      <x:c r="J5" s="7" t="s">
         <x:v>263</x:v>
-      </x:c>
-      <x:c r="J5" s="7" t="s">
-        <x:v>264</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A6" s="7" t="s">
+        <x:v>264</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>265</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>266</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
         <x:v>121</x:v>
@@ -2585,7 +2582,7 @@
       </x:c>
       <x:c r="E6" s="7"/>
       <x:c r="F6" s="7" t="s">
-        <x:v>267</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="G6" s="7" t="s">
         <x:v>90</x:v>
@@ -2595,7 +2592,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J6" s="7" t="s">
-        <x:v>268</x:v>
+        <x:v>267</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="17" customHeight="1">
@@ -2621,7 +2618,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="7" t="s">
-        <x:v>269</x:v>
+        <x:v>268</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="17" customHeight="1">
@@ -2809,7 +2806,7 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>270</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -2906,15 +2903,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="7" t="s">
-        <x:v>271</x:v>
+        <x:v>270</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A5" s="7" t="s">
+        <x:v>271</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>272</x:v>
-      </x:c>
-      <x:c r="B5" s="7" t="s">
-        <x:v>273</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
         <x:v>95</x:v>
@@ -2927,18 +2924,18 @@
       <x:c r="G5" s="7"/>
       <x:c r="H5" s="7"/>
       <x:c r="I5" s="8" t="s">
+        <x:v>273</x:v>
+      </x:c>
+      <x:c r="J5" s="7" t="s">
         <x:v>274</x:v>
-      </x:c>
-      <x:c r="J5" s="7" t="s">
-        <x:v>275</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A6" s="7" t="s">
+        <x:v>275</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>276</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>277</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
         <x:v>95</x:v>
@@ -2953,18 +2950,18 @@
       </x:c>
       <x:c r="H6" s="7"/>
       <x:c r="I6" s="8" t="s">
+        <x:v>277</x:v>
+      </x:c>
+      <x:c r="J6" s="7" t="s">
         <x:v>278</x:v>
-      </x:c>
-      <x:c r="J6" s="7" t="s">
-        <x:v>279</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A7" s="7" t="s">
+        <x:v>279</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>280</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="s">
-        <x:v>281</x:v>
       </x:c>
       <x:c r="C7" s="7" t="s">
         <x:v>121</x:v>
@@ -2982,15 +2979,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J7" s="7" t="s">
-        <x:v>282</x:v>
+        <x:v>281</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A8" s="7" t="s">
+        <x:v>282</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>283</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="s">
-        <x:v>284</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
         <x:v>149</x:v>
@@ -3006,18 +3003,18 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="J8" s="7" t="s">
-        <x:v>285</x:v>
+        <x:v>284</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A9" s="7" t="s">
+        <x:v>285</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>286</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>287</x:v>
-      </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D9" s="7"/>
       <x:c r="E9" s="7"/>
@@ -3027,18 +3024,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I9" s="8" t="s">
+        <x:v>287</x:v>
+      </x:c>
+      <x:c r="J9" s="7" t="s">
         <x:v>288</x:v>
-      </x:c>
-      <x:c r="J9" s="7" t="s">
-        <x:v>289</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A10" s="7" t="s">
+        <x:v>289</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>290</x:v>
-      </x:c>
-      <x:c r="B10" s="7" t="s">
-        <x:v>291</x:v>
       </x:c>
       <x:c r="C10" s="7" t="s">
         <x:v>206</x:v>
@@ -3051,18 +3048,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I10" s="8" t="s">
+        <x:v>291</x:v>
+      </x:c>
+      <x:c r="J10" s="7" t="s">
         <x:v>292</x:v>
-      </x:c>
-      <x:c r="J10" s="7" t="s">
-        <x:v>293</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A11" s="7" t="s">
+        <x:v>293</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>294</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="s">
-        <x:v>295</x:v>
       </x:c>
       <x:c r="C11" s="7" t="s">
         <x:v>206</x:v>
@@ -3075,18 +3072,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I11" s="8" t="s">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="J11" s="7" t="s">
         <x:v>296</x:v>
-      </x:c>
-      <x:c r="J11" s="7" t="s">
-        <x:v>297</x:v>
       </x:c>
     </x:row>
     <x:row r="12" s="1" customFormat="1">
       <x:c r="A12" s="9" t="s">
+        <x:v>297</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="s">
         <x:v>298</x:v>
-      </x:c>
-      <x:c r="B12" s="9" t="s">
-        <x:v>299</x:v>
       </x:c>
       <x:c r="C12" s="9" t="s">
         <x:v>95</x:v>
@@ -3099,10 +3096,10 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I12" s="9" t="s">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="J12" s="9" t="s">
         <x:v>300</x:v>
-      </x:c>
-      <x:c r="J12" s="9" t="s">
-        <x:v>301</x:v>
       </x:c>
     </x:row>
     <x:row r="13" s="1" customFormat="1">
@@ -3128,7 +3125,7 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="J13" s="9" t="s">
-        <x:v>302</x:v>
+        <x:v>301</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3158,7 +3155,7 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>303</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -3255,7 +3252,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="7" t="s">
-        <x:v>304</x:v>
+        <x:v>303</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="17" customHeight="1">
@@ -3281,18 +3278,18 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="J5" s="7" t="s">
-        <x:v>305</x:v>
+        <x:v>304</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A6" s="7" t="s">
+        <x:v>305</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>306</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>307</x:v>
-      </x:c>
       <x:c r="C6" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
         <x:v>90</x:v>
@@ -3301,13 +3298,13 @@
       <x:c r="F6" s="7"/>
       <x:c r="G6" s="7"/>
       <x:c r="H6" s="7" t="s">
-        <x:v>308</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="I6" s="8" t="s">
         <x:v>96</x:v>
       </x:c>
       <x:c r="J6" s="7" t="s">
-        <x:v>309</x:v>
+        <x:v>308</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="17" customHeight="1">
@@ -3331,18 +3328,18 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="J7" s="7" t="s">
-        <x:v>310</x:v>
+        <x:v>309</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A8" s="7" t="s">
+        <x:v>310</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>311</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="s">
+      <x:c r="C8" s="7" t="s">
         <x:v>312</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="s">
-        <x:v>313</x:v>
       </x:c>
       <x:c r="D8" s="7" t="s">
         <x:v>90</x:v>
@@ -3352,21 +3349,21 @@
       <x:c r="G8" s="7"/>
       <x:c r="H8" s="7"/>
       <x:c r="I8" s="8" t="s">
+        <x:v>313</x:v>
+      </x:c>
+      <x:c r="J8" s="7" t="s">
         <x:v>314</x:v>
-      </x:c>
-      <x:c r="J8" s="7" t="s">
-        <x:v>315</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A9" s="7" t="s">
+        <x:v>315</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>316</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>317</x:v>
-      </x:c>
       <x:c r="C9" s="7" t="s">
-        <x:v>313</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="D9" s="7" t="s">
         <x:v>90</x:v>
@@ -3376,21 +3373,21 @@
       <x:c r="G9" s="7"/>
       <x:c r="H9" s="7"/>
       <x:c r="I9" s="8" t="s">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c r="J9" s="7" t="s">
         <x:v>318</x:v>
-      </x:c>
-      <x:c r="J9" s="7" t="s">
-        <x:v>319</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A10" s="7" t="s">
+        <x:v>319</x:v>
+      </x:c>
+      <x:c r="B10" s="7" t="s">
         <x:v>320</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="s">
-        <x:v>321</x:v>
-      </x:c>
       <x:c r="C10" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D10" s="7"/>
       <x:c r="E10" s="7"/>
@@ -3400,21 +3397,21 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I10" s="8" t="s">
+        <x:v>321</x:v>
+      </x:c>
+      <x:c r="J10" s="7" t="s">
         <x:v>322</x:v>
-      </x:c>
-      <x:c r="J10" s="7" t="s">
-        <x:v>323</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A11" s="7" t="s">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>324</x:v>
       </x:c>
-      <x:c r="B11" s="7" t="s">
-        <x:v>325</x:v>
-      </x:c>
       <x:c r="C11" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D11" s="7"/>
       <x:c r="E11" s="7" t="s">
@@ -3428,18 +3425,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I11" s="8" t="s">
+        <x:v>325</x:v>
+      </x:c>
+      <x:c r="J11" s="7" t="s">
         <x:v>326</x:v>
-      </x:c>
-      <x:c r="J11" s="7" t="s">
-        <x:v>327</x:v>
       </x:c>
     </x:row>
     <x:row r="12" s="1" customFormat="1">
       <x:c r="A12" s="9" t="s">
+        <x:v>327</x:v>
+      </x:c>
+      <x:c r="B12" s="9" t="s">
         <x:v>328</x:v>
-      </x:c>
-      <x:c r="B12" s="9" t="s">
-        <x:v>329</x:v>
       </x:c>
       <x:c r="C12" s="9" t="s">
         <x:v>30</x:v>
@@ -3455,15 +3452,15 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="J12" s="9" t="s">
-        <x:v>330</x:v>
+        <x:v>329</x:v>
       </x:c>
     </x:row>
     <x:row r="13" s="1" customFormat="1">
       <x:c r="A13" s="9" t="s">
+        <x:v>330</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="s">
         <x:v>331</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="s">
-        <x:v>332</x:v>
       </x:c>
       <x:c r="C13" s="9" t="s">
         <x:v>30</x:v>
@@ -3476,18 +3473,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I13" s="9" t="s">
+        <x:v>332</x:v>
+      </x:c>
+      <x:c r="J13" s="9" t="s">
         <x:v>333</x:v>
-      </x:c>
-      <x:c r="J13" s="9" t="s">
-        <x:v>334</x:v>
       </x:c>
     </x:row>
     <x:row r="14" s="1" customFormat="1">
       <x:c r="A14" s="9" t="s">
+        <x:v>334</x:v>
+      </x:c>
+      <x:c r="B14" s="9" t="s">
         <x:v>335</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="s">
-        <x:v>336</x:v>
       </x:c>
       <x:c r="C14" s="9" t="s">
         <x:v>30</x:v>
@@ -3500,18 +3497,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I14" s="9" t="s">
+        <x:v>336</x:v>
+      </x:c>
+      <x:c r="J14" s="9" t="s">
         <x:v>337</x:v>
-      </x:c>
-      <x:c r="J14" s="9" t="s">
-        <x:v>338</x:v>
       </x:c>
     </x:row>
     <x:row r="15" s="1" customFormat="1">
       <x:c r="A15" s="9" t="s">
+        <x:v>338</x:v>
+      </x:c>
+      <x:c r="B15" s="9" t="s">
         <x:v>339</x:v>
-      </x:c>
-      <x:c r="B15" s="9" t="s">
-        <x:v>340</x:v>
       </x:c>
       <x:c r="C15" s="9" t="s">
         <x:v>186</x:v>
@@ -3529,18 +3526,18 @@
         <x:v>3600</x:v>
       </x:c>
       <x:c r="J15" s="9" t="s">
-        <x:v>341</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="16" s="1" customFormat="1">
       <x:c r="A16" s="9" t="s">
-        <x:v>342</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="B16" s="9" t="s">
-        <x:v>299</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="C16" s="9" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D16" s="9"/>
       <x:c r="E16" s="9"/>
@@ -3550,18 +3547,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I16" s="9" t="s">
+        <x:v>342</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="s">
         <x:v>343</x:v>
-      </x:c>
-      <x:c r="J16" s="9" t="s">
-        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="1" customFormat="1">
       <x:c r="A17" s="9" t="s">
+        <x:v>344</x:v>
+      </x:c>
+      <x:c r="B17" s="9" t="s">
         <x:v>345</x:v>
-      </x:c>
-      <x:c r="B17" s="9" t="s">
-        <x:v>346</x:v>
       </x:c>
       <x:c r="C17" s="9" t="s">
         <x:v>206</x:v>
@@ -3574,10 +3571,10 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I17" s="9" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="J17" s="9" t="s">
         <x:v>347</x:v>
-      </x:c>
-      <x:c r="J17" s="9" t="s">
-        <x:v>348</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="1" customFormat="1">
@@ -3605,7 +3602,7 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="J18" s="9" t="s">
-        <x:v>349</x:v>
+        <x:v>348</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3635,7 +3632,7 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>350</x:v>
+        <x:v>349</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -3736,15 +3733,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="7" t="s">
-        <x:v>351</x:v>
+        <x:v>350</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A5" s="7" t="s">
+        <x:v>351</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>352</x:v>
-      </x:c>
-      <x:c r="B5" s="7" t="s">
-        <x:v>353</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
         <x:v>149</x:v>
@@ -3756,21 +3753,21 @@
       <x:c r="F5" s="7"/>
       <x:c r="G5" s="7"/>
       <x:c r="H5" s="7" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="I5" s="8" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="J5" s="7" t="s">
         <x:v>354</x:v>
-      </x:c>
-      <x:c r="I5" s="8" t="s">
-        <x:v>354</x:v>
-      </x:c>
-      <x:c r="J5" s="7" t="s">
-        <x:v>355</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A6" s="7" t="s">
+        <x:v>355</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>356</x:v>
-      </x:c>
-      <x:c r="B6" s="7" t="s">
-        <x:v>357</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
         <x:v>186</x:v>
@@ -3788,15 +3785,15 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="J6" s="7" t="s">
-        <x:v>358</x:v>
+        <x:v>357</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A7" s="7" t="s">
+        <x:v>358</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>359</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="s">
-        <x:v>360</x:v>
       </x:c>
       <x:c r="C7" s="7" t="s">
         <x:v>104</x:v>
@@ -3811,7 +3808,7 @@
         <x:v>light</x:v>
       </x:c>
       <x:c r="I7" s="8" t="s">
-        <x:v>361</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
         <x:v>外观模式，当前仅支持浅色。</x:v>
@@ -3886,7 +3883,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
-        <x:v>362</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="C11" s="7" t="s">
         <x:v>162</x:v>
@@ -3908,7 +3905,7 @@
         <x:v>114</x:v>
       </x:c>
       <x:c r="J11" s="7" t="s">
-        <x:v>363</x:v>
+        <x:v>362</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3938,34 +3935,34 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="B1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="C1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="D1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="E1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="F1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="G1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="H1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="I1" s="4" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
       <x:c r="J1" s="5" t="s">
-        <x:v>364</x:v>
+        <x:v>363</x:v>
       </x:c>
     </x:row>
     <x:row r="2" s="1" customFormat="1" ht="17" customHeight="1">
@@ -4032,10 +4029,10 @@
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A4" s="7" t="s">
+        <x:v>364</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="s">
         <x:v>365</x:v>
-      </x:c>
-      <x:c r="B4" s="7" t="s">
-        <x:v>366</x:v>
       </x:c>
       <x:c r="C4" s="7" t="s">
         <x:v>121</x:v>
@@ -4055,18 +4052,18 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="7" t="s">
-        <x:v>367</x:v>
+        <x:v>366</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A5" s="7" t="s">
-        <x:v>368</x:v>
+        <x:v>367</x:v>
       </x:c>
       <x:c r="B5" s="7" t="s">
         <x:v>176</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
-        <x:v>313</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="D5" s="7" t="s">
         <x:v>90</x:v>
@@ -4076,21 +4073,21 @@
       <x:c r="G5" s="7"/>
       <x:c r="H5" s="7"/>
       <x:c r="I5" s="8" t="s">
+        <x:v>368</x:v>
+      </x:c>
+      <x:c r="J5" s="7" t="s">
         <x:v>369</x:v>
-      </x:c>
-      <x:c r="J5" s="7" t="s">
-        <x:v>370</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A6" s="7" t="s">
+        <x:v>370</x:v>
+      </x:c>
+      <x:c r="B6" s="7" t="s">
         <x:v>371</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="s">
+      <x:c r="C6" s="7" t="s">
         <x:v>372</x:v>
-      </x:c>
-      <x:c r="C6" s="7" t="s">
-        <x:v>373</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
         <x:v>90</x:v>
@@ -4100,15 +4097,15 @@
       <x:c r="G6" s="7"/>
       <x:c r="H6" s="7"/>
       <x:c r="I6" s="8" t="s">
+        <x:v>373</x:v>
+      </x:c>
+      <x:c r="J6" s="7" t="s">
         <x:v>374</x:v>
-      </x:c>
-      <x:c r="J6" s="7" t="s">
-        <x:v>375</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A7" s="7" t="s">
-        <x:v>376</x:v>
+        <x:v>375</x:v>
       </x:c>
       <x:c r="B7" s="7" t="s">
         <x:v>148</x:v>
@@ -4124,7 +4121,7 @@
       <x:c r="G7" s="7"/>
       <x:c r="H7" s="7"/>
       <x:c r="I7" s="8" t="s">
-        <x:v>377</x:v>
+        <x:v>376</x:v>
       </x:c>
       <x:c r="J7" s="7" t="str">
         <x:v>消息正文，最长 1000 个字符。</x:v>
@@ -4132,10 +4129,10 @@
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A8" s="7" t="s">
+        <x:v>377</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>378</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="s">
-        <x:v>379</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
         <x:v>149</x:v>
@@ -4148,18 +4145,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I8" s="8" t="s">
-        <x:v>354</x:v>
+        <x:v>353</x:v>
       </x:c>
       <x:c r="J8" s="7" t="s">
-        <x:v>380</x:v>
+        <x:v>379</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A9" s="7" t="s">
+        <x:v>380</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>381</x:v>
-      </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>382</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
         <x:v>30</x:v>
@@ -4174,10 +4171,10 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I9" s="8" t="s">
+        <x:v>382</x:v>
+      </x:c>
+      <x:c r="J9" s="7" t="s">
         <x:v>383</x:v>
-      </x:c>
-      <x:c r="J9" s="7" t="s">
-        <x:v>384</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="1" customFormat="1" ht="17" customHeight="1">
@@ -4203,7 +4200,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J10" s="7" t="s">
-        <x:v>385</x:v>
+        <x:v>384</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="1" customFormat="1" ht="17" customHeight="1">
@@ -4256,7 +4253,7 @@
         <x:v>134</x:v>
       </x:c>
       <x:c r="I12" s="8" t="s">
-        <x:v>383</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="J12" s="7" t="s">
         <x:v>136</x:v>
@@ -4282,7 +4279,7 @@
         <x:v>134</x:v>
       </x:c>
       <x:c r="I13" s="8" t="s">
-        <x:v>383</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="J13" s="7" t="s">
         <x:v>139</x:v>
@@ -4492,7 +4489,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re63836892bf74abf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R788f66b8ccf94cd4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6282,23 +6279,27 @@
       <x:c r="D6" s="7" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="E6" s="7"/>
+      <x:c r="E6" s="7" t="str">
+        <x:v>是</x:v>
+      </x:c>
       <x:c r="F6" s="7"/>
-      <x:c r="G6" s="7"/>
+      <x:c r="G6" s="7" t="str">
+        <x:v>是</x:v>
+      </x:c>
       <x:c r="H6" s="7"/>
       <x:c r="I6" s="8" t="s">
         <x:v>207</x:v>
       </x:c>
-      <x:c r="J6" s="7" t="s">
-        <x:v>208</x:v>
+      <x:c r="J6" s="7" t="str">
+        <x:v>工单问题描述；有效数据（is_deleted = 0）按 md5(problem_desc) 唯一。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A7" s="7" t="s">
+        <x:v>208</x:v>
+      </x:c>
+      <x:c r="B7" s="7" t="s">
         <x:v>209</x:v>
-      </x:c>
-      <x:c r="B7" s="7" t="s">
-        <x:v>210</x:v>
       </x:c>
       <x:c r="C7" s="7" t="s">
         <x:v>206</x:v>
@@ -6311,18 +6312,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I7" s="8" t="s">
+        <x:v>210</x:v>
+      </x:c>
+      <x:c r="J7" s="7" t="s">
         <x:v>211</x:v>
-      </x:c>
-      <x:c r="J7" s="7" t="s">
-        <x:v>212</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A8" s="7" t="s">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="B8" s="7" t="s">
         <x:v>213</x:v>
-      </x:c>
-      <x:c r="B8" s="7" t="s">
-        <x:v>214</x:v>
       </x:c>
       <x:c r="C8" s="7" t="s">
         <x:v>121</x:v>
@@ -6342,15 +6343,15 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J8" s="7" t="s">
-        <x:v>215</x:v>
+        <x:v>214</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A9" s="7" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B9" s="7" t="s">
         <x:v>216</x:v>
-      </x:c>
-      <x:c r="B9" s="7" t="s">
-        <x:v>217</x:v>
       </x:c>
       <x:c r="C9" s="7" t="s">
         <x:v>113</x:v>
@@ -6368,7 +6369,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>217</x:v>
       </x:c>
     </x:row>
     <x:row r="10" s="1" customFormat="1" ht="17" customHeight="1">
@@ -6396,15 +6397,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J10" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>218</x:v>
       </x:c>
     </x:row>
     <x:row r="11" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A11" s="7" t="s">
+        <x:v>219</x:v>
+      </x:c>
+      <x:c r="B11" s="7" t="s">
         <x:v>220</x:v>
-      </x:c>
-      <x:c r="B11" s="7" t="s">
-        <x:v>221</x:v>
       </x:c>
       <x:c r="C11" s="7" t="s">
         <x:v>113</x:v>
@@ -6422,15 +6423,15 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J11" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>221</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="17">
       <x:c r="A12" s="7" t="s">
+        <x:v>222</x:v>
+      </x:c>
+      <x:c r="B12" s="7" t="s">
         <x:v>223</x:v>
-      </x:c>
-      <x:c r="B12" s="7" t="s">
-        <x:v>224</x:v>
       </x:c>
       <x:c r="C12" s="7" t="s">
         <x:v>30</x:v>
@@ -6443,18 +6444,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I12" s="8" t="s">
+        <x:v>224</x:v>
+      </x:c>
+      <x:c r="J12" s="7" t="s">
         <x:v>225</x:v>
-      </x:c>
-      <x:c r="J12" s="7" t="s">
-        <x:v>226</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="9" t="s">
+        <x:v>226</x:v>
+      </x:c>
+      <x:c r="B13" s="9" t="s">
         <x:v>227</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="s">
-        <x:v>228</x:v>
       </x:c>
       <x:c r="C13" s="9" t="s">
         <x:v>30</x:v>
@@ -6467,18 +6468,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I13" s="9" t="s">
-        <x:v>225</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="J13" s="9" t="s">
-        <x:v>229</x:v>
+        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="9" t="s">
+        <x:v>229</x:v>
+      </x:c>
+      <x:c r="B14" s="9" t="s">
         <x:v>230</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="s">
-        <x:v>231</x:v>
       </x:c>
       <x:c r="C14" s="9" t="s">
         <x:v>30</x:v>
@@ -6491,18 +6492,18 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="I14" s="9" t="s">
+        <x:v>231</x:v>
+      </x:c>
+      <x:c r="J14" s="9" t="s">
         <x:v>232</x:v>
-      </x:c>
-      <x:c r="J14" s="9" t="s">
-        <x:v>233</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="9" t="s">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c r="B15" s="9" t="s">
         <x:v>234</x:v>
-      </x:c>
-      <x:c r="B15" s="9" t="s">
-        <x:v>235</x:v>
       </x:c>
       <x:c r="C15" s="9" t="s">
         <x:v>95</x:v>
@@ -6515,21 +6516,21 @@
       <x:c r="G15" s="9"/>
       <x:c r="H15" s="9"/>
       <x:c r="I15" s="9" t="s">
+        <x:v>235</x:v>
+      </x:c>
+      <x:c r="J15" s="9" t="s">
         <x:v>236</x:v>
-      </x:c>
-      <x:c r="J15" s="9" t="s">
-        <x:v>237</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="9" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="B16" s="9" t="s">
         <x:v>238</x:v>
       </x:c>
-      <x:c r="B16" s="9" t="s">
+      <x:c r="C16" s="9" t="s">
         <x:v>239</x:v>
-      </x:c>
-      <x:c r="C16" s="9" t="s">
-        <x:v>240</x:v>
       </x:c>
       <x:c r="D16" s="9" t="s">
         <x:v>90</x:v>
@@ -6539,18 +6540,18 @@
       <x:c r="G16" s="9"/>
       <x:c r="H16" s="9"/>
       <x:c r="I16" s="9" t="s">
+        <x:v>240</x:v>
+      </x:c>
+      <x:c r="J16" s="9" t="s">
         <x:v>241</x:v>
-      </x:c>
-      <x:c r="J16" s="9" t="s">
-        <x:v>242</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="9" t="s">
+        <x:v>242</x:v>
+      </x:c>
+      <x:c r="B17" s="9" t="s">
         <x:v>243</x:v>
-      </x:c>
-      <x:c r="B17" s="9" t="s">
-        <x:v>244</x:v>
       </x:c>
       <x:c r="C17" s="9" t="s">
         <x:v>30</x:v>
@@ -6563,10 +6564,10 @@
       <x:c r="G17" s="9"/>
       <x:c r="H17" s="9"/>
       <x:c r="I17" s="9" t="s">
+        <x:v>244</x:v>
+      </x:c>
+      <x:c r="J17" s="9" t="s">
         <x:v>245</x:v>
-      </x:c>
-      <x:c r="J17" s="9" t="s">
-        <x:v>246</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -6728,7 +6729,7 @@
   <x:sheetData>
     <x:row r="1" s="1" customFormat="1">
       <x:c r="A1" s="3" t="s">
-        <x:v>247</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -6804,7 +6805,7 @@
     </x:row>
     <x:row r="4" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A4" s="7" t="s">
-        <x:v>248</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="B4" s="7" t="s">
         <x:v>142</x:v>
@@ -6824,18 +6825,18 @@
       </x:c>
       <x:c r="H4" s="7"/>
       <x:c r="I4" s="8" t="s">
+        <x:v>248</x:v>
+      </x:c>
+      <x:c r="J4" s="7" t="s">
         <x:v>249</x:v>
-      </x:c>
-      <x:c r="J4" s="7" t="s">
-        <x:v>250</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A5" s="7" t="s">
+        <x:v>250</x:v>
+      </x:c>
+      <x:c r="B5" s="7" t="s">
         <x:v>251</x:v>
-      </x:c>
-      <x:c r="B5" s="7" t="s">
-        <x:v>252</x:v>
       </x:c>
       <x:c r="C5" s="7" t="s">
         <x:v>104</x:v>
@@ -6852,21 +6853,21 @@
       </x:c>
       <x:c r="H5" s="7"/>
       <x:c r="I5" s="8" t="s">
+        <x:v>252</x:v>
+      </x:c>
+      <x:c r="J5" s="7" t="s">
         <x:v>253</x:v>
-      </x:c>
-      <x:c r="J5" s="7" t="s">
-        <x:v>254</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="1" customFormat="1" ht="17" customHeight="1">
       <x:c r="A6" s="7" t="s">
-        <x:v>255</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="B6" s="7" t="s">
         <x:v>145</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="D6" s="7" t="s">
         <x:v>90</x:v>
@@ -6876,10 +6877,10 @@
       <x:c r="G6" s="7"/>
       <x:c r="H6" s="7"/>
       <x:c r="I6" s="8" t="s">
+        <x:v>255</x:v>
+      </x:c>
+      <x:c r="J6" s="7" t="s">
         <x:v>256</x:v>
-      </x:c>
-      <x:c r="J6" s="7" t="s">
-        <x:v>257</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="1" customFormat="1" ht="17" customHeight="1">

</xml_diff>